<commit_message>
feat: T088 Model 1 / Fix 1.2b — ballistic kettlebell lifts on new Layout 10 (bell ladder)
KB swings/snatches/cleans/jerks are trained for high-power reps at a bell, not a
1RM. Tagged 13 ballistic KB moves lift_type=ballistic. New BallisticLiftDetail
(mobile) + AdminStrengthBallisticDetail (web mirror): bell-ladder strip + next-bell
hero + StrongFirst/S&S/snatch-test cue. Dispatch routes ballistic before the
weighted branch. Layout 10 added to the catalog + CLAUDE.md spec. Completes Model 1.
</commit_message>
<xml_diff>
--- a/docs/Layout Design.xlsx
+++ b/docs/Layout Design.xlsx
@@ -821,13 +821,42 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="1" t="n"/>
-      <c r="B11" s="1" t="n"/>
-      <c r="C11" s="1" t="n"/>
-      <c r="D11" s="1" t="n"/>
-      <c r="E11" s="1" t="n"/>
-      <c r="F11" s="1" t="n"/>
-      <c r="G11" s="1" t="n"/>
+      <c r="A11" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Strength</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>Ballistic (kettlebell)</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>Bell-ladder strip
+Hero card (next bell)
+Chart and log
+(no swipe pill, no rep-max grid)</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>For ballistic kettlebell lifts (swing / snatch / clean / jerk / push-press / high-pull) trained for high-power reps, NOT a 1RM. Progression is a bell ladder — own a bell at a clean rep volume, then size up. Benchmarks: Simple &amp; Sinister, the snatch test.</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>Kettlebell Swing, Kettlebell Snatch, Kettlebell Clean and Jerk, Double Kettlebell Swing, Single Arm Kettlebell Swing</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>Grind kettlebell moves (Strict Press, Front Squat, Deadlift, Turkish Get-Up, Windmill) stay on Layout 3 (weighted).</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="n"/>

</xml_diff>

<commit_message>
feat: T088 Model 3 leverage family — skill holds on new Layout 11 (leverage ladder)
Planche/levers/flag/handstand/etc. fail on leverage, not endurance — a 2-min
planche grid is meaningless. Added movements.hold_type (time/load/leverage),
tagged 18 leverage holds. New LeverageHoldDetail (mobile) + AdminStrengthLeverageDetail
(web mirror): short 5-30s milestones + a skill ladder (tuck->straddle->full, 30s
clean -> next variant), standalone holds chase the 30s mastered mark. Dispatch
routes leverage before the isometric branch. Layout 11 in catalog + CLAUDE.md;
iso spec updated to exclude leverage. Load family (add-load holds) still pending.
</commit_message>
<xml_diff>
--- a/docs/Layout Design.xlsx
+++ b/docs/Layout Design.xlsx
@@ -859,13 +859,42 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="1" t="n"/>
-      <c r="B12" s="1" t="n"/>
-      <c r="C12" s="1" t="n"/>
-      <c r="D12" s="1" t="n"/>
-      <c r="E12" s="1" t="n"/>
-      <c r="F12" s="1" t="n"/>
-      <c r="G12" s="1" t="n"/>
+      <c r="A12" s="3" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Strength</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>Leverage / skill hold (isometric)</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>Skill-ladder strip (variants)
+Short milestone tiles (5-30s)
+Hero (hold target / progress-to-next)
+Chart and log</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>For skill/leverage isometric holds (planche, front/back lever, human flag, L-sit, handstand, crow, support holds). They fail on leverage, not endurance — a full planche maxes ~10-20s — so short milestones (5-30s) + a variant ladder (tuck -&gt; straddle -&gt; full) replace the 10-120s time grid. Hold 30s clean -&gt; progress to the next variant.</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>Planche Hold (Tuck), Front Lever Hold, Human Flag Hold, Handstand Hold (Wall)</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="inlineStr">
+        <is>
+          <t>Standalone holds (no harder variant in the app) just chase the 30s 'mastered' mark. hold_type='leverage'. Loadable holds (hold_type='load') are a separate planned treatment.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="n"/>

</xml_diff>

<commit_message>
feat: T088 Model 3 load family — loadable holds on new Layout 12 (build then add load)
Wall sit, calf-raise/glute-bridge holds, dead hang, etc. take external load, so
grinding to 2 min trains endurance not strength. Tagged 7 holds hold_type='load'.
New LoadHoldDetail (mobile) + AdminStrengthLoadDetail (web mirror): phase 1 builds
the bodyweight hold to 60s (time milestones), phase 2 adds load (5lb/2.5kg steps,
~30s target). Iso log form gains an optional Added-weight wheel for load-holds
(label "Name · W unit x D sec"; value stays "D sec"). Chart adaptive (load once
weighted, else time). Dispatch before isometric. Layout 12 + CLAUDE.md + iso spec.
Model 3 complete (time/leverage/load all handled).
</commit_message>
<xml_diff>
--- a/docs/Layout Design.xlsx
+++ b/docs/Layout Design.xlsx
@@ -897,13 +897,41 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="1" t="n"/>
-      <c r="B13" s="1" t="n"/>
-      <c r="C13" s="1" t="n"/>
-      <c r="D13" s="1" t="n"/>
-      <c r="E13" s="1" t="n"/>
-      <c r="F13" s="1" t="n"/>
-      <c r="G13" s="1" t="n"/>
+      <c r="A13" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Strength</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>Loadable hold (isometric)</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>Time milestone tiles (15-60s)
+Hero (build-to-60s -&gt; add-load)
+Chart and log</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>For loadable isometric holds (wall sit, calf-raise hold, glute-bridge holds, dead hang, split-squat hold, squat hold). Build the bodyweight hold to ~60s, THEN add external load — grinding to 2 min trains endurance, not strength. Two phases: time milestones (15-60s) -&gt; an add-load progression.</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>Wall Sit, Calf Raise Hold, Glute Bridge Hold, Dead Hang, Split Squat Hold</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>hold_type='load'. Athlete log form gains an optional Added-weight wheel; label 'Name · 25 lb x 45 sec', value stays '45 sec'. Chart shows load once weighted, else hold time. Coach mirror is read-only (no log).</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="n"/>

</xml_diff>

<commit_message>
fix: bodyweight chart splits per assist tier (T088 round-2 #4)
The Pull-Up / bodyweight consolidated chart blended every assist tier onto
one curve (e.g. 13 light-band reps next to 5 full-RX reps), which misreads as
a single progression. Now the chart filters to the ACTIVE tier (the pill you
are on) so each tier gets its own line; the personal-best reference line and
caption follow the active tier and re-filter on pill swipe. Mobile + web
mirror + CLAUDE.md BW spec + Layout Design.xlsx + T088 ledger.
</commit_message>
<xml_diff>
--- a/docs/Layout Design.xlsx
+++ b/docs/Layout Design.xlsx
@@ -533,7 +533,8 @@
           <t>Page swipe pill
 10 tile 5-5 grid
 Hero card
-Consolidated chart and log</t>
+Per-tier chart (one curve per pill)
+Shared log</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
@@ -546,7 +547,11 @@
           <t>Pull Up, Push Up, Dip</t>
         </is>
       </c>
-      <c r="G2" s="3" t="n"/>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>Round-2 #4: progress chart is PER-TIER (filters to the active pill's tier) - was wrongly blending band-assisted reps with full-RX reps on one curve.</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="43.2" customHeight="1">
       <c r="A3" s="2" t="n">

</xml_diff>

<commit_message>
feat: swipe-acceptance rule - per-variant elements swipe, shared don't (T089)
Locked rule: on a variant page an element accepts the variant-swipe iff its
content is per-variant; shared/consolidated elements (the log included) don't.
Audited every swipeable surface (2 Explore agents). Carry/Sled/Swimming/Air
Bike/Rucking already compliant; fixed two gaps:
 - Bodyweight chart (per-tier after #4) now accepts the tier-swipe via a Pan +
   a scroll-sync effect in the consolidated block so the hero pager follows.
 - Weighted hero gets its own zone-swipe (was pill-only).
Documented as the source of truth in docs/Layout Design.xlsx (per-element
column + global note) and CLAUDE.md (Swipe-acceptance rule section).
</commit_message>
<xml_diff>
--- a/docs/Layout Design.xlsx
+++ b/docs/Layout Design.xlsx
@@ -16,13 +16,17 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00111721"/>
     </font>
   </fonts>
   <fills count="2">
@@ -60,7 +64,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -69,6 +73,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -466,7 +474,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G15"/>
+  <dimension ref="A1:H17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="8.21875" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -475,6 +483,7 @@
     <col width="33.5546875" customWidth="1" min="5" max="5"/>
     <col width="24.109375" customWidth="1" min="6" max="6"/>
     <col width="68.33203125" bestFit="1" customWidth="1" min="7" max="7"/>
+    <col width="60" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -511,6 +520,11 @@
       <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Issues</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Swipe rule (per element; LOCKED 2026-06-05)</t>
         </is>
       </c>
     </row>
@@ -552,6 +566,11 @@
           <t>Round-2 #4: progress chart is PER-TIER (filters to the active pill's tier) - was wrongly blending band-assisted reps with full-RX reps on one curve.</t>
         </is>
       </c>
+      <c r="H2" s="4" t="inlineStr">
+        <is>
+          <t>VARIANT = assist tier. Swipe: pill, hero, tiles, chart (all per-tier). Log does NOT swipe (consolidated across tiers, with tier chips).</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="43.2" customHeight="1">
       <c r="A3" s="2" t="n">
@@ -585,6 +604,11 @@
         </is>
       </c>
       <c r="G3" s="3" t="n"/>
+      <c r="H3" s="4" t="inlineStr">
+        <is>
+          <t>No variant swipe (single variant; tap milestone tiles).</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="72" customHeight="1">
       <c r="A4" s="2" t="n">
@@ -619,6 +643,11 @@
         </is>
       </c>
       <c r="G4" s="3" t="n"/>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>VARIANT = adp zone. Swipe: pill, hero (per-zone). Tiles SCROLL (shared 1-15RM grid). Chart + log do NOT swipe (shared across zones).</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="57.6" customHeight="1">
       <c r="A5" s="2" t="n">
@@ -652,6 +681,11 @@
         </is>
       </c>
       <c r="G5" s="3" t="n"/>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>VARIANT = adp zone. Swipe: pill, hero (per-zone, paged). Chart + log do NOT swipe (shared across zones).</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="57.6" customHeight="1">
       <c r="A6" s="2" t="n">
@@ -686,6 +720,11 @@
         </is>
       </c>
       <c r="G6" s="3" t="n"/>
+      <c r="H6" s="4" t="inlineStr">
+        <is>
+          <t>VARIANT = sub-variant (Push/Pull). WHOLE page per-variant: pill, hero, chart, log ALL swipe (each filtered to the active variant).</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="57.6" customHeight="1">
       <c r="A7" s="2" t="n">
@@ -720,6 +759,11 @@
         </is>
       </c>
       <c r="G7" s="3" t="n"/>
+      <c r="H7" s="4" t="inlineStr">
+        <is>
+          <t>VARIANT = stroke. WHOLE page per-variant: pill, hero, plan tiles, chart, log ALL swipe (each filtered to the active stroke).</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="57.6" customHeight="1">
       <c r="A8" s="2" t="n">
@@ -753,6 +797,11 @@
         </is>
       </c>
       <c r="G8" s="3" t="n"/>
+      <c r="H8" s="4" t="inlineStr">
+        <is>
+          <t>No variant swipe (single variant; tap plan tiles).</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="43.2" customHeight="1">
       <c r="A9" s="2" t="n">
@@ -786,6 +835,11 @@
         </is>
       </c>
       <c r="G9" s="3" t="n"/>
+      <c r="H9" s="4" t="inlineStr">
+        <is>
+          <t>No variant swipe (single variant; tap rep tiles).</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="n">
@@ -824,6 +878,11 @@
           <t>Ballistic kettlebell moves (swing/snatch) are rep-based, NOT %-of-1RM — deferred to a separate rep-based treatment (Fix 1.2b).</t>
         </is>
       </c>
+      <c r="H10" s="4" t="inlineStr">
+        <is>
+          <t>No variant swipe (tap the 3 intensity tiles).</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="n">
@@ -862,6 +921,11 @@
           <t>Grind kettlebell moves (Strict Press, Front Squat, Deadlift, Turkish Get-Up, Windmill) stay on Layout 3 (weighted).</t>
         </is>
       </c>
+      <c r="H11" s="4" t="inlineStr">
+        <is>
+          <t>No variant swipe (single bell ladder; tap).</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="n">
@@ -900,6 +964,11 @@
           <t>Standalone holds (no harder variant in the app) just chase the 30s 'mastered' mark. hold_type='leverage'. Loadable holds (hold_type='load') are a separate planned treatment.</t>
         </is>
       </c>
+      <c r="H12" s="4" t="inlineStr">
+        <is>
+          <t>Per-variant skill ladder. Currently tap; round-2 #5 will consolidate to the swimming pattern -&gt; then pill+hero+chart+log all per-variant swipe.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="n">
@@ -935,6 +1004,11 @@
       <c r="G13" s="3" t="inlineStr">
         <is>
           <t>hold_type='load'. Athlete log form gains an optional Added-weight wheel; label 'Name · 25 lb x 45 sec', value stays '45 sec'. Chart shows load once weighted, else hold time. Coach mirror is read-only (no log).</t>
+        </is>
+      </c>
+      <c r="H13" s="4" t="inlineStr">
+        <is>
+          <t>No variant swipe today (single variant; tap). Round-2 #6 rebuild keeps it single-variant (TUT tile grid).</t>
         </is>
       </c>
     </row>
@@ -956,7 +1030,24 @@
       <c r="F15" s="1" t="n"/>
       <c r="G15" s="1" t="n"/>
     </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>SWIPE-ACCEPTANCE RULE (LOCKED 2026-06-05)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="120" customHeight="1">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>On a variant page, an element accepts the variant-swipe gesture IF AND ONLY IF its content is per-variant (it changes when you swipe to another variant). A shared / consolidated element (same content across all variants) does NOT swipe -- it scrolls / taps / reads normally. The discriminator is one question: 'is this element's content shared across variants?' -&gt; shared = no swipe, not-shared = swipe. This applies element by element, the LOG included: a per-variant (filtered) log swipes (e.g. Sled, Swimming); a consolidated log does not (e.g. Bodyweight tiers). Likewise a per-variant chart swipes (Bodyweight after the per-tier split, Sled, Swimming) but a chart that is shared across zones does not (Weighted, Carry, Air Bike, Rucking).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A17:H17"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: load-hold web mirror + web tile-overflow guard (finish T088 #6 end-to-end)
Web side of the two mobile tasks:
 - #6 load-hold: rewrote AdminStrengthLoadDetail to mirror the new mobile view
   (Rohmert-curve projected added-weight per TUT tile, like Pull-Up Full RX;
   title no longer "Add load"; attribution = Rohmert/Oranchuk/ACSM).
 - layout-overflow: added whitespace-nowrap to the web tile values on the
   bodyweight / weighted / Olympic mirrors (prevents the "-> N" push value from
   wrapping). Web plate rows were already safe (flex-wrap + CSS default shrink),
   unlike RN. Cardio audited clean.
Specs: CLAUDE.md Layout-12 + Layout Design.xlsx + T088 ledger (#6 done).
</commit_message>
<xml_diff>
--- a/docs/Layout Design.xlsx
+++ b/docs/Layout Design.xlsx
@@ -986,8 +986,8 @@
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>Time milestone tiles (15-60s)
-Hero (build-to-60s -&gt; add-load)
+          <t>TUT tile grid (10-90s, projected +weight per tile)
+Hero (selected-tile target + cue)
 Chart and log</t>
         </is>
       </c>
@@ -1003,7 +1003,7 @@
       </c>
       <c r="G13" s="3" t="inlineStr">
         <is>
-          <t>hold_type='load'. Athlete log form gains an optional Added-weight wheel; label 'Name · 25 lb x 45 sec', value stays '45 sec'. Chart shows load once weighted, else hold time. Coach mirror is read-only (no log).</t>
+          <t>hold_type='load'. Round-2 #6 rebuild: tiles PROJECT added weight per duration via Rohmert's isometric-endurance curve (like Pull-Up Full RX); 'Add load' removed as the card title (now in the cue); attribution = Rohmert/Oranchuk/ACSM. Athlete log form has an Added-weight wheel; web mirror is read-only.</t>
         </is>
       </c>
       <c r="H13" s="4" t="inlineStr">

</xml_diff>

<commit_message>
docs: lock leverage family consolidation (T088 round-2 #5)
CLAUDE.md Layout-11 spec rewritten with the Family-consolidation block + the
mobile generic-engine dispatch order; Layout Design.xlsx row 11 moved to the
DONE/consolidated state (variant pill + per-variant slots, web shows variants
individually); TASK_PIPELINE ledger marks round-2 #5 + the overarching swimming
pass done for strength (leverage was the last true multi-variant strength family).
</commit_message>
<xml_diff>
--- a/docs/Layout Design.xlsx
+++ b/docs/Layout Design.xlsx
@@ -943,30 +943,30 @@
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>Skill-ladder strip (variants)
+          <t>Page swipe pill (variant family)
 Short milestone tiles (5-30s)
 Hero (hold target / progress-to-next)
-Chart and log</t>
+Per-variant chart and log</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>For skill/leverage isometric holds (planche, front/back lever, human flag, L-sit, handstand, crow, support holds). They fail on leverage, not endurance — a full planche maxes ~10-20s — so short milestones (5-30s) + a variant ladder (tuck -&gt; straddle -&gt; full) replace the 10-120s time grid. Hold 30s clean -&gt; progress to the next variant.</t>
+          <t>For skill/leverage isometric holds (planche, front/back lever, human flag, L-sit, handstand, crow, support holds). They fail on leverage, not endurance - a full planche maxes ~10-20s - so short milestones (5-30s) + a variant ladder (tuck -&gt; straddle -&gt; full) replace the 10-120s time grid. Hold 30s clean -&gt; progress to the next variant. The 4 multi-variant families consolidate through the GENERIC family engine (same as Sled/Swimming); standalone holds are single-variant.</t>
         </is>
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>Planche Hold (Tuck), Front Lever Hold, Human Flag Hold, Handstand Hold (Wall)</t>
+          <t>Planche Hold [Tuck/Straddle/Full], Front Lever Hold [Tuck/Full], Back Lever Hold [Tuck/Full], Handstand Hold [Wall/Freestanding]; standalone: L-Sit, V-Sit, Human Flag, Headstand, Crow</t>
         </is>
       </c>
       <c r="G12" s="3" t="inlineStr">
         <is>
-          <t>Standalone holds (no harder variant in the app) just chase the 30s 'mastered' mark. hold_type='leverage'. Loadable holds (hold_type='load') are a separate planned treatment.</t>
+          <t>hold_type='leverage'. June 2026 DB migration renamed variants to 'Name [Variant]' bracket form + linked them to a parent container (parent_movement_id + variant_short_label) so the generic FamilyConsolidatedDetail renders them. Standalone holds (no harder variant) chase the 30s 'mastered' mark with no pill. Loadable holds (hold_type='load') = Layout 12.</t>
         </is>
       </c>
       <c r="H12" s="4" t="inlineStr">
         <is>
-          <t>Per-variant skill ladder. Currently tap; round-2 #5 will consolidate to the swimming pattern -&gt; then pill+hero+chart+log all per-variant swipe.</t>
+          <t>DONE round-2 #5: the 4 multi-variant families consolidate via the GENERIC engine (variant pill + paged per-variant slots). WHOLE page per-variant on mobile: pill, hero, milestone tiles, chart, log ALL swipe (each slot is a full per-variant skill-hold page). Standalone holds = single variant, no pill (tap tiles). Web coach view shows variants individually (no web generic engine; pill carousel deferred).</t>
         </is>
       </c>
     </row>

</xml_diff>